<commit_message>
feat(firmas): celular opcional en la firma (columna 'Celular en firma'), icono de telefono y fix de saltos de linea en version texto
</commit_message>
<xml_diff>
--- a/_generador-firmas/plantilla-personas.xlsx
+++ b/_generador-firmas/plantilla-personas.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2000"/>
+  <dimension ref="A1:I2000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -445,8 +445,9 @@
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="52" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -482,11 +483,16 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Celular en firma</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Incluir</t>
         </is>
       </c>
@@ -6490,7 +6496,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Elegí Sí o No" type="list">
+    <dataValidation sqref="G2:G2000 I2:I2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Elegí Sí o No" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6504,7 +6510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -6562,22 +6568,29 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
+          <t>Celular en firma (opcional): Sí para mostrar el celular en la firma, con su ícono. Vacío o No: la firma no lo muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
           <t>LinkedIn (opcional): URL del perfil. Si queda vacío, la firma no muestra LinkedIn.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Incluir (opcional): No para excluir a la persona sin borrar la fila. Vacío equivale a Sí.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr"/>
-    </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Esta planilla tiene datos personales: no la subas al repositorio ni la compartas fuera de la empresa.</t>
         </is>

</xml_diff>